<commit_message>
Combination drug now allwos for randomizer
</commit_message>
<xml_diff>
--- a/CQ_Plate/CQ_InputTemplate.xlsx
+++ b/CQ_Plate/CQ_InputTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebas\Documents\GitHub\ot2\CQ_Plate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jornb\Documents\GitHub\ot2-JB\upstream (R) processors\CQ_Plate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E3E6A4-9205-4E8A-815D-240FD9C36C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10A42BC6-B5A2-412F-93BB-106ACCD94F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="61">
   <si>
     <t>Drug Name</t>
   </si>
@@ -239,6 +239,9 @@
   </si>
   <si>
     <t>&gt;No underscores!</t>
+  </si>
+  <si>
+    <t>&gt;For controls that you don’t want to randomize use "control" or "ctrl"</t>
   </si>
 </sst>
 </file>
@@ -368,7 +371,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -384,9 +387,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -424,7 +427,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -530,7 +533,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -672,7 +675,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -681,14 +684,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O64"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.73046875" customWidth="1"/>
-    <col min="4" max="4" width="9.73046875" customWidth="1"/>
-    <col min="15" max="15" width="63.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.77734375" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" customWidth="1"/>
+    <col min="15" max="15" width="63.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
@@ -710,7 +713,7 @@
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -735,7 +738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
@@ -760,12 +763,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="O4" s="8">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
@@ -780,7 +783,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
@@ -801,20 +804,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H7" s="8"/>
       <c r="O7" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="12.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>4</v>
       </c>
       <c r="H8" s="8"/>
       <c r="O8" s="8"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B9" s="1">
         <v>1</v>
       </c>
@@ -852,7 +855,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -872,7 +875,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -912,7 +915,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -949,7 +952,7 @@
       </c>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
@@ -986,7 +989,7 @@
       </c>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
@@ -1023,7 +1026,7 @@
       </c>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -1060,7 +1063,7 @@
       </c>
       <c r="M15" s="2"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
@@ -1097,7 +1100,7 @@
       </c>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>12</v>
       </c>
@@ -1114,12 +1117,12 @@
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B20" s="1">
         <v>1</v>
       </c>
@@ -1157,7 +1160,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>5</v>
       </c>
@@ -1201,7 +1204,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -1245,7 +1248,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>7</v>
       </c>
@@ -1286,7 +1289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
@@ -1327,7 +1330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>9</v>
       </c>
@@ -1368,7 +1371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
@@ -1409,7 +1412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -1450,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>12</v>
       </c>
@@ -1491,12 +1494,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B32" s="1">
         <v>1</v>
       </c>
@@ -1534,7 +1537,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>5</v>
       </c>
@@ -1578,7 +1581,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -1622,7 +1625,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>7</v>
       </c>
@@ -1663,7 +1666,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>8</v>
       </c>
@@ -1704,7 +1707,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>9</v>
       </c>
@@ -1745,7 +1748,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>10</v>
       </c>
@@ -1786,7 +1789,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
@@ -1827,7 +1830,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -1868,12 +1871,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B44" s="1">
         <v>1</v>
       </c>
@@ -1911,7 +1914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="45" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>5</v>
       </c>
@@ -1931,7 +1934,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="15.75" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>6</v>
       </c>
@@ -1971,7 +1974,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="47" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>7</v>
       </c>
@@ -2011,7 +2014,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="48" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -2051,7 +2054,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>9</v>
       </c>
@@ -2083,8 +2086,11 @@
       </c>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="O49" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>10</v>
       </c>
@@ -2117,7 +2123,7 @@
       <c r="L50" s="2"/>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>11</v>
       </c>
@@ -2150,7 +2156,7 @@
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
@@ -2167,12 +2173,12 @@
       <c r="L52" s="2"/>
       <c r="M52" s="2"/>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B56" s="1">
         <v>1</v>
       </c>
@@ -2210,7 +2216,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>5</v>
       </c>
@@ -2263,7 +2269,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>6</v>
       </c>
@@ -2316,7 +2322,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>7</v>
       </c>
@@ -2369,7 +2375,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>8</v>
       </c>
@@ -2422,7 +2428,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>9</v>
       </c>
@@ -2475,7 +2481,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>10</v>
       </c>
@@ -2528,7 +2534,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>11</v>
       </c>
@@ -2581,7 +2587,7 @@
         <v xml:space="preserve"> 0 MED-A </v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>12</v>
       </c>
@@ -2643,4 +2649,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d465f887-04a9-4c17-8b62-103eddccf68b}" enabled="1" method="Standard" siteId="{ca2a7f76-dbd7-4ec0-9108-6b3d524fb7c8}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>